<commit_message>
1. streamline the resource usage
</commit_message>
<xml_diff>
--- a/src/scraping/data/cold_start/argos.xlsx
+++ b/src/scraping/data/cold_start/argos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kumo/programming/competitor_product_search/src/scraping/data/cold_start/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02181464-27B4-E245-9518-EBC6E4FF53ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5242D44F-939E-714C-B2C1-4442F451D392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7020" yWindow="24300" windowWidth="24280" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3140" yWindow="1440" windowWidth="24280" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cold_start" sheetId="1" r:id="rId1"/>
@@ -46,22 +46,23 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
+    <t>https://www.argos.co.uk/product/7726851</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.argos.co.uk/product/8463948</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.argos.co.uk/product/7662881</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.argos.co.uk/product/tuc148159202</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
     <t>https://www.argos.co.uk/product/8695390</t>
-  </si>
-  <si>
-    <t>https://www.argos.co.uk/product/7726851</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.argos.co.uk/product/8463948</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.argos.co.uk/product/7662881</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.argos.co.uk/product/tuc148159202</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -427,7 +428,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="22" customHeight="1">
@@ -435,7 +436,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -443,7 +444,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -451,7 +452,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -459,7 +460,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -475,6 +476,7 @@
     <hyperlink ref="B4" r:id="rId3" xr:uid="{77B6E916-A06D-1940-B2A7-0A22CA250942}"/>
     <hyperlink ref="B6" r:id="rId4" xr:uid="{AF9AF725-C755-7742-BCE9-FBA35D704675}"/>
     <hyperlink ref="B7" r:id="rId5" xr:uid="{26158707-C5EA-7C45-BE29-93F80F863C85}"/>
+    <hyperlink ref="B5" r:id="rId6" xr:uid="{8BD393ED-DCFA-7748-B9EA-9EC3963078E4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>